<commit_message>
teste mudei o preço do café para 1000€
</commit_message>
<xml_diff>
--- a/Preços P7.xlsx
+++ b/Preços P7.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matil\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matil\Desktop\menu-posto-7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D14B2B-7140-45A5-B853-E3EEE5329E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40105C7-4540-48F5-805A-86E54177DCD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1165,7 +1165,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1]"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1176,22 +1176,26 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -1200,6 +1204,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1222,7 +1233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1252,6 +1263,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1525,7 +1539,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="6">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>10</v>
@@ -1547,7 +1561,7 @@
       <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="11">
         <v>2</v>
       </c>
       <c r="F4" s="5" t="s">

</xml_diff>

<commit_message>
tentar meter de novo como estava
</commit_message>
<xml_diff>
--- a/Preços P7.xlsx
+++ b/Preços P7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matil\Desktop\menu-posto-7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40105C7-4540-48F5-805A-86E54177DCD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0FD685-1A12-4B62-B41A-7BC0A38AA4DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1165,7 +1165,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1]"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1205,13 +1205,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1233,7 +1226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1263,9 +1256,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1539,7 +1529,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="6">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>10</v>
@@ -1561,7 +1551,7 @@
       <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="4">
         <v>2</v>
       </c>
       <c r="F4" s="5" t="s">

</xml_diff>